<commit_message>
Phase 4 steps 4-6: switching and routing pages on a shared family template
Shared card builder, filter engine, family panels, selectors, compare rows and value labels;
FamilyPage/ModelRow/ModelDetail/SelectorPage/ComparePage take a family; compare gains ?f=;
hub selector shortcut offers one selector per family; TR/EN strings and 9 glossary terms added.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/catalog/routing.xlsx
+++ b/data/catalog/routing.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5866" uniqueCount="1461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5867" uniqueCount="1461">
   <si>
     <t>family</t>
   </si>
@@ -2756,7 +2756,7 @@
     <t>2031-11-30</t>
   </si>
   <si>
-    <t>Cisco'nun önerdiği yedek: C8111-C-G2-MX (Meraki yönetimli Catalyst 8111-G2).</t>
+    <t>Cisco'nun önerdiği yedek: Meraki yönetimli Catalyst 8111 G2 yönlendirici (henüz kataloğa eklenmedi).</t>
   </si>
   <si>
     <t>https://www.cisco.com/c/en/us/products/collateral/security/meraki-cloud-managed-security-appliances/mx67c-mx68cw-eol.pdf</t>
@@ -2837,7 +2837,7 @@
     <t>Meraki MX68 cloud-managed security appliance (end of sale announced): 3 WAN ports (up to 1G); stateful firewall 700 Mbps, next-generation firewall (NGFW) 400 Mbps. Built-in cellular (LTE/5G) modem. Supports SD-WAN. Has ports that can supply PoE.</t>
   </si>
   <si>
-    <t>Cisco'nun önerdiği yedek: C8121-CW-G2-MX (Meraki yönetimli Catalyst 8121-G2).</t>
+    <t>Cisco'nun önerdiği yedek: Meraki yönetimli Catalyst 8121 G2 yönlendirici (henüz kataloğa eklenmedi).</t>
   </si>
   <si>
     <t>wireless, lte, poe, cryptography, ngfw_capable, ips, ids, advanced_malware_protection, url_filtering</t>
@@ -3161,7 +3161,7 @@
     <t>2029-09-04</t>
   </si>
   <si>
-    <t>Yedek olarak Z4 / Z4C öneriliyor; ikisi de henüz yayınlanmadı (veri eksik).</t>
+    <t>Yedek olarak yeni nesil Z-Series geçidi öneriliyor (henüz kataloğa eklenmedi).</t>
   </si>
   <si>
     <t>https://documentation.meraki.com/@api/deki/files/24994/Z3-HW_EOS_Notice_(1).pdf?revision=1</t>
@@ -3200,7 +3200,10 @@
     <t>Meraki Z-Series teleworker gateway (end of sale): 2 WAN ports (up to 1G); stateful firewall 100 Mbps. Built-in cellular (LTE/5G) modem. Supports SD-WAN. Has ports that can supply PoE.</t>
   </si>
   <si>
-    <t>Yedek olarak Z4C öneriliyor; henüz yayınlanmadı (veri eksik). Z3C-HW-WW için son sipariş 11 Şubat 2024'tü.</t>
+    <t>Z4C</t>
+  </si>
+  <si>
+    <t>Z3C-HW-WW için son sipariş 11 Şubat 2024'tü.</t>
   </si>
   <si>
     <t>https://documentation.meraki.com/@api/deki/files/24993/Z3C-HW-NA.pdf?revision=1</t>
@@ -3239,9 +3242,6 @@
     <t>The Z4 datasheet page could not be read (the specs are not in the page text); Z4C was read and Z4 is not assumed to match it.</t>
   </si>
   <si>
-    <t>Z4C</t>
-  </si>
-  <si>
     <t>Meraki Z-Series uzaktan çalışan geçidi: 2 WAN portu (en fazla 1G); durum izlemeli güvenlik duvarı 500 Mbps, güvenlik 300 Mbps. Dahili hücresel (LTE/5G) modem. SD-WAN destekler. PoE verebilen portları var.</t>
   </si>
   <si>
@@ -4388,10 +4388,10 @@
     <t>Meraki MX95: a firewall and SD-WAN appliance managed from the Meraki dashboard, for large branches and small campuses.</t>
   </si>
   <si>
-    <t>Meraki Z-Series: uzaktan çalışanlar için küçük, bulut yönetimli güvenlik geçidi; evden şirket ağına VPN kurar. Burada Z4C ile satışı sona eren Z3 modelleri listelenir; Z4 henüz eklenmedi.</t>
-  </si>
-  <si>
-    <t>Meraki Z-Series: small cloud-managed security gateways for teleworkers that build a VPN from home to the company network. Listed here are the Z4C and the Z3 models, which are end of sale; the Z4 is not added yet.</t>
+    <t>Meraki Z-Series: uzaktan çalışanlar için küçük, bulut yönetimli güvenlik geçidi; evden şirket ağına VPN kurar. Burada Z4C ile satışı sona eren Z3 modelleri listelenir; diğer Z-Series modelleri henüz eklenmedi.</t>
+  </si>
+  <si>
+    <t>Meraki Z-Series: small cloud-managed security gateways for teleworkers that build a VPN from home to the company network. Listed here are the Z4C and the Z3 models, which are end of sale; the other Z-Series models are not added yet.</t>
   </si>
   <si>
     <t>Meraki vMX: AWS, Azure, Google Cloud ve Alibaba Cloud'da çalışan sanal MX; bulut kaynaklarını Meraki SD-WAN ağına bağlar. S, M ve L boyutları vardır.</t>
@@ -21134,12 +21134,14 @@
       <c r="O117" s="1" t="s">
         <v>1047</v>
       </c>
-      <c r="P117" s="1"/>
+      <c r="P117" s="1" t="s">
+        <v>1061</v>
+      </c>
       <c r="Q117" s="1" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="S117" s="1" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="T117" t="s">
         <v>55</v>
@@ -21159,7 +21161,7 @@
         <v>1052</v>
       </c>
       <c r="AA117" s="1" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="AB117" s="1" t="s">
         <v>345</v>
@@ -21218,25 +21220,25 @@
         <v>291</v>
       </c>
       <c r="AZ117" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="BA117" s="1" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="BB117" s="1" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="BC117" s="1" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="BD117" s="1" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="BE117" s="1"/>
     </row>
     <row r="118" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="B118" t="s">
         <v>76</v>
@@ -21251,10 +21253,10 @@
         <v>28</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G118" s="1" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="H118" s="1"/>
       <c r="I118" s="1"/>
@@ -21274,7 +21276,7 @@
       <c r="X118" s="1"/>
       <c r="Y118" s="1"/>
       <c r="Z118" s="1" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="AA118" s="1"/>
       <c r="AB118" s="1"/>
@@ -21333,24 +21335,24 @@
         <v>1053</v>
       </c>
       <c r="BA118" s="1" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="BB118" s="1" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="BC118" s="1" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="BD118" s="1" t="s">
         <v>1057</v>
       </c>
       <c r="BE118" s="1" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="119" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
-        <v>1074</v>
+        <v>1061</v>
       </c>
       <c r="B119" t="s">
         <v>76</v>
@@ -21365,10 +21367,10 @@
         <v>28</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>1074</v>
+        <v>1061</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>1074</v>
+        <v>1061</v>
       </c>
       <c r="H119" s="1" t="s">
         <v>1075</v>
@@ -21471,7 +21473,7 @@
         <v>291</v>
       </c>
       <c r="AZ119" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="BA119" s="1" t="s">
         <v>1080</v>
@@ -21483,7 +21485,7 @@
         <v>1082</v>
       </c>
       <c r="BD119" s="1" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="BE119" s="1"/>
     </row>

</xml_diff>